<commit_message>
update LWC module as per report analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org_LWC.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org_LWC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FrameworkProjectAutomationCode\govgrants-framework-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05EDAF15-AB71-42A9-B6E5-A7560ABB96F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC31142-AC19-4F2A-A931-C670FF632431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7940" yWindow="2810" windowWidth="11260" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="1" r:id="rId1"/>
@@ -43,9 +43,6 @@
     <t>ProgramName__c</t>
   </si>
   <si>
-    <t>Automation Internal Program for Testing</t>
-  </si>
-  <si>
     <t>fieldType__c</t>
   </si>
   <si>
@@ -77,6 +74,9 @@
   </si>
   <si>
     <t>fieldObjectives__c</t>
+  </si>
+  <si>
+    <t>Automation Program For Test</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -442,10 +442,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -453,10 +453,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -464,10 +464,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -475,10 +475,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -512,7 +512,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -523,7 +523,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>1825</v>
@@ -534,10 +534,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -545,10 +545,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor and update LWC test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_QA_org_LWC.xlsx
+++ b/src/main/resources/Program_Field_Values_QA_org_LWC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FrameworkProjectAutomationCode\govgrants-framework-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC31142-AC19-4F2A-A931-C670FF632431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65F9480-3494-488C-9ECD-F49391AD4CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7940" yWindow="2810" windowWidth="11260" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProgramCreation_v" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -77,6 +77,15 @@
   </si>
   <si>
     <t>Automation Program For Test</t>
+  </si>
+  <si>
+    <t>fieldDeadlines__c</t>
+  </si>
+  <si>
+    <t>Test field description deadline</t>
+  </si>
+  <si>
+    <t>Test Descrption1</t>
   </si>
 </sst>
 </file>
@@ -488,12 +497,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E38D00-D360-40DE-A015-68B4C19080CD}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -548,7 +557,18 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>